<commit_message>
update template daily plan
</commit_message>
<xml_diff>
--- a/Template/template_daily_plan.xlsx
+++ b/Template/template_daily_plan.xlsx
@@ -5,7 +5,7 @@
   <workbookPr defaultThemeVersion="164011"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\DIGITALISASI\PROJECT IP\1. Document &amp; Files\Excel\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\xampp\htdocs\iphylon\Template\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
@@ -537,7 +537,7 @@
         <v>8</v>
       </c>
       <c r="B7" s="4">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="8" spans="1:30" x14ac:dyDescent="0.25">
@@ -851,7 +851,7 @@
         <v>8</v>
       </c>
       <c r="B14" s="4">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="15" spans="1:30" x14ac:dyDescent="0.25">
@@ -1103,11 +1103,11 @@
       <c r="AD19" s="8"/>
     </row>
     <row r="20" spans="1:30" x14ac:dyDescent="0.25">
-      <c r="A20" s="9" t="s">
+      <c r="A20" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="B20" s="1">
-        <v>3</v>
+      <c r="B20" s="4">
+        <v>2</v>
       </c>
     </row>
     <row r="21" spans="1:30" x14ac:dyDescent="0.25">

</xml_diff>